<commit_message>
CD-197: Disallow STX FISH image submissions to ENA
</commit_message>
<xml_diff>
--- a/images/stx_fish_image_schema_main_v0.1.xlsx
+++ b/images/stx_fish_image_schema_main_v0.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Documents/EI/Projects/COPO-schemas/images/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D215CBE6-07FA-1D44-8A6B-A6890E63F3B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F37A50B-A3A7-CB49-B686-660649BABCF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32740" yWindow="-940" windowWidth="30240" windowHeight="17900" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
+    <workbookView xWindow="37500" yWindow="-320" windowWidth="30240" windowHeight="17900" activeTab="3" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="413">
   <si>
     <t>component_name</t>
   </si>
@@ -6985,9 +6985,6 @@
       <c r="B2" t="s">
         <v>240</v>
       </c>
-      <c r="C2" t="s">
-        <v>17</v>
-      </c>
       <c r="D2" t="s">
         <v>17</v>
       </c>

</xml_diff>